<commit_message>
feat: support secondary barcode in product import and export
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/import_productos.xlsx
+++ b/public/templates/import_productos.xlsx
@@ -397,20 +397,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,36 +419,39 @@
         <v>codigo_barra</v>
       </c>
       <c r="B1" t="str">
+        <v>codigo_barra_secundario</v>
+      </c>
+      <c r="C1" t="str">
         <v>nombre</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>unidad_medida</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>factor_pack</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>precio_costo</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>precio_venta</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>margen</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>categoria</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>proveedor</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>area_fisica</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>stock_inicial</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>activo</v>
       </c>
     </row>
@@ -456,42 +460,45 @@
         <v>7790001000101</v>
       </c>
       <c r="B2" t="str">
+        <v>7790001000102</v>
+      </c>
+      <c r="C2" t="str">
         <v>Coca Cola 500ml</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>pack</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>6</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>1200</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>1800</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>50</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>Bebidas</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Distribuidora Sur</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>Góndola 1</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>10</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>SI</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>